<commit_message>
updated averages for female1 and male1 data
</commit_message>
<xml_diff>
--- a/Models/CLIP/female1data/clip_big5_female1_have_jewerly.xlsx
+++ b/Models/CLIP/female1data/clip_big5_female1_have_jewerly.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tamucs-my.sharepoint.com/personal/yq_c_tamu_edu/Documents/Research/genderBias/GenderBias-SRL-Implementation/Models/CLIP/female1data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_EACEDFC023065587DC4467CB1F3182828CBC3968" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EF6864F-81F8-434A-AD87-76A1E56EF14C}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Extraversion" sheetId="1" r:id="rId1"/>
@@ -13,12 +19,25 @@
     <sheet name="Neuroticism" sheetId="4" r:id="rId4"/>
     <sheet name="Openness" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="48">
   <si>
     <t>Positive Trait</t>
   </si>
@@ -159,14 +178,25 @@
   </si>
   <si>
     <t>Likes to reflect, play with ideas</t>
+  </si>
+  <si>
+    <t>avg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -194,21 +224,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -246,7 +285,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -280,6 +319,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -314,9 +354,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -489,11 +530,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,62 +552,75 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.04436862096190453</v>
+        <v>4.4368620961904533E-2</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
       </c>
       <c r="D2">
-        <v>0.01719256862998009</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>1.7192568629980091E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3">
-        <v>0.03241653740406036</v>
+        <v>3.2416537404060357E-2</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
       <c r="D3">
-        <v>0.003464081091806293</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>3.464081091806293E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0.01252174098044634</v>
+        <v>1.252174098044634E-2</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
       </c>
       <c r="D4">
-        <v>0.0008944204309955239</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>8.9442043099552393E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5">
-        <v>0.008760293945670128</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>8.7602939456701279E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0.00417989818379283</v>
+        <v>4.1798981837928304E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="1">
+        <f>AVERAGE(B2:B6)</f>
+        <v>2.0449418295174836E-2</v>
+      </c>
+      <c r="D7" s="1">
+        <f>AVERAGE(D2:D6)</f>
+        <v>7.1836900509273027E-3</v>
       </c>
     </row>
   </sheetData>
@@ -571,11 +629,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="37" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -589,68 +651,81 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2">
-        <v>0.04072697460651398</v>
+        <v>4.0726974606513977E-2</v>
       </c>
       <c r="C2" t="s">
         <v>17</v>
       </c>
       <c r="D2">
-        <v>0.015573900192976</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>1.5573900192976E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3">
-        <v>0.01018820330500603</v>
+        <v>1.0188203305006031E-2</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
       </c>
       <c r="D3">
-        <v>0.009764950722455978</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>9.7649507224559784E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4">
-        <v>0.009614072740077972</v>
+        <v>9.6140727400779724E-3</v>
       </c>
       <c r="C4" t="s">
         <v>19</v>
       </c>
       <c r="D4">
-        <v>0.004601652268320322</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>4.601652268320322E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
       <c r="B5">
-        <v>0.006115449592471123</v>
+        <v>6.1154495924711227E-3</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
       </c>
       <c r="D5">
-        <v>0.001711975084617734</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>1.711975084617734E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
       <c r="B6">
-        <v>0.004928798414766788</v>
+        <v>4.9287984147667876E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="1">
+        <f>AVERAGE(B2:B6)</f>
+        <v>1.4314699731767178E-2</v>
+      </c>
+      <c r="D7" s="1">
+        <f>AVERAGE(D2:D6)</f>
+        <v>7.9131195670925081E-3</v>
       </c>
     </row>
   </sheetData>
@@ -659,11 +734,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="37.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.08984375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -677,68 +756,81 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
       <c r="B2">
-        <v>0.02863724902272224</v>
+        <v>2.8637249022722241E-2</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
       </c>
       <c r="D2">
-        <v>0.005463826004415751</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>5.4638260044157514E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>22</v>
       </c>
       <c r="B3">
-        <v>0.02116590365767479</v>
+        <v>2.1165903657674789E-2</v>
       </c>
       <c r="C3" t="s">
         <v>27</v>
       </c>
       <c r="D3">
-        <v>0.003107172902673483</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>3.1071729026734829E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>23</v>
       </c>
       <c r="B4">
-        <v>0.003593332367017865</v>
+        <v>3.5933323670178652E-3</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
       </c>
       <c r="D4">
-        <v>0.00129983841907233</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>1.29983841907233E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
       <c r="B5">
-        <v>0.002295271493494511</v>
+        <v>2.2952714934945111E-3</v>
       </c>
       <c r="C5" t="s">
         <v>29</v>
       </c>
       <c r="D5">
-        <v>0.0008926274604164064</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>8.9262746041640639E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>25</v>
       </c>
       <c r="B6">
-        <v>0.001293741399422288</v>
+        <v>1.2937413994222879E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="1">
+        <f>AVERAGE(B2:B6)</f>
+        <v>1.1397099588066339E-2</v>
+      </c>
+      <c r="D7" s="1">
+        <f>AVERAGE(D2:D6)</f>
+        <v>2.6908661966444924E-3</v>
       </c>
     </row>
   </sheetData>
@@ -747,11 +839,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="32.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -765,62 +861,75 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>30</v>
       </c>
       <c r="B2">
-        <v>0.03963758051395416</v>
+        <v>3.9637580513954163E-2</v>
       </c>
       <c r="C2" t="s">
         <v>33</v>
       </c>
       <c r="D2">
-        <v>0.007673930376768112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>7.6739303767681122E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>31</v>
       </c>
       <c r="B3">
-        <v>0.02060496807098389</v>
+        <v>2.060496807098389E-2</v>
       </c>
       <c r="C3" t="s">
         <v>34</v>
       </c>
       <c r="D3">
-        <v>0.004205143544822931</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>4.2051435448229313E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>32</v>
       </c>
       <c r="B4">
-        <v>0.008228389546275139</v>
+        <v>8.2283895462751389E-3</v>
       </c>
       <c r="C4" t="s">
         <v>35</v>
       </c>
       <c r="D4">
-        <v>0.00391809269785881</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>3.9180926978588104E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>36</v>
       </c>
       <c r="D5">
-        <v>0.00317209679633379</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>3.1720967963337898E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>37</v>
       </c>
       <c r="D6">
-        <v>0.003001923440024257</v>
+        <v>3.0019234400242571E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="1">
+        <f>AVERAGE(B2:B6)</f>
+        <v>2.2823646043737728E-2</v>
+      </c>
+      <c r="D7" s="1">
+        <f>AVERAGE(D2:D6)</f>
+        <v>4.3942373711615803E-3</v>
       </c>
     </row>
   </sheetData>
@@ -829,11 +938,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="35.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -847,72 +960,85 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>38</v>
       </c>
       <c r="B2">
-        <v>0.3025061190128326</v>
+        <v>0.30250611901283259</v>
       </c>
       <c r="C2" t="s">
         <v>45</v>
       </c>
       <c r="D2">
-        <v>0.1527748852968216</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>0.15277488529682159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>39</v>
       </c>
       <c r="B3">
-        <v>0.06009076908230782</v>
+        <v>6.0090769082307822E-2</v>
       </c>
       <c r="C3" t="s">
         <v>46</v>
       </c>
       <c r="D3">
-        <v>0.01223496440798044</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>1.223496440798044E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>40</v>
       </c>
       <c r="B4">
-        <v>0.04568222165107727</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+        <v>4.5682221651077271E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>41</v>
       </c>
       <c r="B5">
-        <v>0.02395028248429298</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+        <v>2.3950282484292981E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>42</v>
       </c>
       <c r="B6">
-        <v>0.01425490714609623</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+        <v>1.425490714609623E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>43</v>
       </c>
       <c r="B7">
-        <v>0.001880846684798598</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>1.8808466847985981E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>44</v>
       </c>
       <c r="B8">
-        <v>0.001409766846336424</v>
+        <v>1.4097668463364239E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="1">
+        <f>AVERAGE(B2:B8)</f>
+        <v>6.4253558986820267E-2</v>
+      </c>
+      <c r="D9" s="1">
+        <f>AVERAGE(D2:D8)</f>
+        <v>8.2504924852401018E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>